<commit_message>
feat(workbook): Preparation sheet only with pre-mixes; Round 6 sample rebuilt
- compact(): the Preparation sheet, its navigation line and its tab link
  only when the Round has (portioned) pre-mixes; sheet_navigation() names
  the tabs actually there. PREPARATION_SHEET_EMPTY and SHEET_NAVIGATION
  retired.
- prepare_import(): a workbook with or without Preparation is read; an
  older one with an empty Preparation sheet still uploads.
- build.py: write_round6_results() builds "Round 6 results (pilot).xlsx"
  from the current compact workbook (Round overview + Results), the
  pilot's Round 6 ratings and notes unchanged; the shipped file is
  regenerated with it. The two shipped project JSONs are byte-identical
  to a rebuild, so sample_projects._SUPERSEDED needs no new hash.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/yogurt_pilot/Round 6 results (pilot).xlsx
+++ b/data/samples/yogurt_pilot/Round 6 results (pilot).xlsx
@@ -8,9 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Round overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Preparation" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Results" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="_FoodOptimizer" sheetId="4" state="veryHidden" r:id="rId4"/>
+    <sheet name="Results" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="_FoodOptimizer" sheetId="3" state="veryHidden" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -544,7 +543,7 @@
     <row r="2" ht="65" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Use the sheet tabs: Round overview → Preparation → Results. Tabs are at the bottom in Excel and at the top in Numbers. Review the plan, prepare each formulation separately, then enter measurements on Results and upload this file in the app.</t>
+          <t>Use the sheet tabs: Round overview → Results. Tabs are at the bottom in Excel and at the top in Numbers. Review the plan, prepare each formulation separately, then enter measurements on Results and upload this file in the app.</t>
         </is>
       </c>
     </row>
@@ -888,11 +887,6 @@
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
-        <is>
-          <t>Preparation</t>
-        </is>
-      </c>
-      <c r="C25" s="14" t="inlineStr">
         <is>
           <t>Results</t>
         </is>
@@ -913,8 +907,7 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A25" location="'Round overview'!A1"/>
-    <hyperlink ref="B25" location="'Preparation'!A1"/>
-    <hyperlink ref="C25" location="'Results'!A1"/>
+    <hyperlink ref="B25" location="'Results'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -922,80 +915,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="58" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Preparation — Pre-mixes for this round</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="65" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Use the sheet tabs: Round overview → Preparation → Results. Tabs are at the bottom in Excel and at the top in Numbers. Prepare pre-mixes with fixed ingredient percentages here. For blends where ingredient amounts vary separately, follow the individual amounts on Round overview.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>No pre-mixes are required. Follow the method on Round overview.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="14" t="inlineStr">
-        <is>
-          <t>Round overview</t>
-        </is>
-      </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>Preparation</t>
-        </is>
-      </c>
-      <c r="C7" s="14" t="inlineStr">
-        <is>
-          <t>Results</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>If a link does not open, select the sheet tab with the same name.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <mergeCells count="1">
-    <mergeCell ref="A2:C2"/>
-  </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="A7" location="'Round overview'!A1"/>
-    <hyperlink ref="B7" location="'Preparation'!A1"/>
-    <hyperlink ref="C7" location="'Results'!A1"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1023,7 +942,7 @@
     <row r="2" ht="65" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Use the sheet tabs: Round overview → Preparation → Results. Tabs are at the bottom in Excel and at the top in Numbers. Each formulation has its own column. Blank means not recorded yet. Enter results, then upload this workbook, check the import and save in the app.</t>
+          <t>Use the sheet tabs: Round overview → Results. Tabs are at the bottom in Excel and at the top in Numbers. Each formulation has its own column. Blank means not recorded yet. Enter results, then upload this workbook, check the import and save in the app.</t>
         </is>
       </c>
     </row>
@@ -1204,6 +1123,8 @@
       <c r="D15" s="15" t="n"/>
       <c r="F15" s="15" t="n"/>
     </row>
+    <row r="16"/>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
@@ -1211,11 +1132,6 @@
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
-        <is>
-          <t>Preparation</t>
-        </is>
-      </c>
-      <c r="D18" s="14" t="inlineStr">
         <is>
           <t>Results</t>
         </is>
@@ -1236,15 +1152,14 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A18" location="'Round overview'!A1"/>
-    <hyperlink ref="B18" location="'Preparation'!A1"/>
-    <hyperlink ref="D18" location="'Results'!A1"/>
+    <hyperlink ref="B18" location="'Results'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
feat(samples): the yogurt pilot's attributes take the paper's names
"Tangy" is now "Tanginess" and "Thickness uniformity" "Uniformity"
(display names only; the CSV columns keep theirs). Both shipped JSONs and
"Round 6 results (pilot).xlsx" are rebuilt: values, notes and amounts
unchanged (checked cell by cell; only the two names differ). The db0d6b7
builds' fingerprints join _SUPERSEDED, so an untouched copy from that
build is replaced on first launch; a changed one is kept. Tests,
docstrings and examples follow.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/yogurt_pilot/Round 6 results (pilot).xlsx
+++ b/data/samples/yogurt_pilot/Round 6 results (pilot).xlsx
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Tangy (/15) · Target 5</t>
+          <t>Tanginess (/15) · Target 5</t>
         </is>
       </c>
       <c r="B9" s="16" t="n">
@@ -1041,7 +1041,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Thickness uniformity (/15) · Target 13</t>
+          <t>Uniformity (/15) · Target 13</t>
         </is>
       </c>
       <c r="B10" s="16" t="n">

</xml_diff>

<commit_message>
chore(sample): describe the pilot's method neutrally
The yogurt pilot no longer names its method or source: Rounds 3-10 are
"chosen by an earlier version of this engine", their notes read
"Engine's pick 3.1", Make a round's caption reads "Chosen by the
engine in the pilot", and the unconfirmed dates are gone. The sample
files are rebuilt (scores unchanged) and the previous ones are listed
in _SUPERSEDED so an untouched copy refreshes.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/yogurt_pilot/Round 6 results (pilot).xlsx
+++ b/data/samples/yogurt_pilot/Round 6 results (pilot).xlsx
@@ -1084,17 +1084,17 @@
       </c>
       <c r="B12" s="17" t="inlineStr">
         <is>
-          <t>Pilot batch 6.1 · EGBO</t>
+          <t>Engine's pick 6.1</t>
         </is>
       </c>
       <c r="D12" s="17" t="inlineStr">
         <is>
-          <t>Pilot batch 6.2 · EGBO</t>
+          <t>Engine's pick 6.2</t>
         </is>
       </c>
       <c r="F12" s="17" t="inlineStr">
         <is>
-          <t>Pilot batch 6.3 · EGBO</t>
+          <t>Engine's pick 6.3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(make a round, workbook): sheets line from the file, optional batch size, Round capitalised
S6 the line under the download names Preparation when the file has it; S14
Optional: scale every formulation to one batch size.; N9 Round capitalised in
every label and the workbook; N10 First 5 formulations explore the allowed
amounts. (rest in ?); N11 Generate first to see suggestions too.; N17 upload
path names the fold. Round 6 sample workbook rebuilt for the new return path.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/yogurt_pilot/Round 6 results (pilot).xlsx
+++ b/data/samples/yogurt_pilot/Round 6 results (pilot).xlsx
@@ -799,7 +799,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Total for this round (g)</t>
+          <t>Total for this Round (g)</t>
         </is>
       </c>
     </row>
@@ -876,7 +876,7 @@
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>Across every formulation; a calculated row's total is what the round comes to, not one weighing.</t>
+          <t>Across every formulation; a calculated row's total is what the Round comes to, not one weighing.</t>
         </is>
       </c>
     </row>

</xml_diff>